<commit_message>
Fill Колоноскопы Excel with 20 real catalog products
Populate 03_PRODUCTS from the category page (20 videocolonoscopes: SonoScape,
Pentax, Olympus, Fujifilm, Aohua) with real specs (tube/distal diameter,
working length, depth of field, view angle). Update hero/expert brand mentions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_kolonoskopy.xlsx
+++ b/medford_kolonoskopy.xlsx
@@ -570,12 +570,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Товары категории</t>
+          <t>Товары категории — реальный каталог medford.ru</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>ПЛЕЙСХОЛДЕРЫ — ждём карточки товаров с medford.ru</t>
+          <t>Заполнено с карточек товаров medford.ru</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Товары, характеристики, цены, наличие, РУ, кейсы</t>
+          <t>Цены (по запросу), наличие, страна, статус РУ, кейсы</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Колоноскопы и видеоколоноскопы для эндоскопических отделений и проктологии: диагностика толстой кишки, биопсия и лечебные манипуляции (полипэктомия, остановка кровотечений). Модели Pentax, Fujinon (Fujifilm), Olympus. Доставка по России, монтаж и ввод в эксплуатацию, обучение персонала, гарантия и сервис. ООО «Медфорд» работает с 2009 года, лицензия Росздравнадзора ФС-99-04-000387 (ТОМИ).</t>
+          <t>Видеоколоноскопы для эндоскопических отделений и проктологии: диагностика толстой кишки, биопсия и лечебные манипуляции (полипэктомия, остановка кровотечений). В каталоге модели SonoScape, Pentax, Olympus, Fujifilm и Aohua. Доставка по России, монтаж и ввод в эксплуатацию, обучение персонала, гарантия и сервис. ООО «Медфорд» работает с 2009 года, лицензия Росздравнадзора ФС-99-04-000387 (ТОМИ).</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Список товаров Bitrix (ожидаются карточки)</t>
+          <t>Список товаров Bitrix (20 позиций)</t>
         </is>
       </c>
     </row>
@@ -2707,33 +2707,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="54" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>03_PRODUCTS — Товары категории (ПЛЕЙСХОЛДЕР)</t>
+          <t>03_PRODUCTS — Товары категории (реальный каталог medford.ru)</t>
         </is>
       </c>
     </row>
@@ -2790,40 +2793,55 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PROPERTY_APPLICATION</t>
+          <t>PROPERTY_TUBE_DIAMETER_MM</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
+          <t>PROPERTY_DISTAL_DIAMETER_MM</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_WORKING_LENGTH_MM</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_DEPTH_OF_FIELD_MM</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_VIEW_ANGLE_DEG</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
           <t>PROPERTY_AVAILABILITY</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>PROPERTY_COUNTRY</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_REG_CERTIFICATE</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_WARRANTY</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_CARD_SPECS</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_CARD_TAGLINE</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_PRICE_REQUEST_TEXT</t>
         </is>
@@ -2840,17 +2858,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>[XML_ID]</t>
+          <t>VIDEOKOLONOSKOP_AOHUA_HD_CL1IL</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>[code]</t>
+          <t>videokolonoskop_aohua_hd_cl1il</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>[Модель товара]</t>
+          <t>Видеоколоноскоп Aohua HD-CL1IL</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2859,74 +2877,2010 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>[URL карточки]</t>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_aohua_hd_cl1il/</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>[бренд]</t>
+          <t>Aohua</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>[тип]</t>
+          <t>Колоноскоп</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>[применение]</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+          <t>12,8</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>1680</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>2-100</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>уточнять</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>[страна]</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>уточнять</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр вводимой трубки, мм: 12,8 | Рабочая длина, мм: 1680 | Глубина резкости, мм: 2-100 | Угол поля зрения, °: 140</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Aohua</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_AOHUA_FHD_CL200JL</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_aohua_fhd_cl200jl</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Aohua FHD-CL200JL</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_aohua_fhd_cl200jl/</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Aohua</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>12,8</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>12,8</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>уточнять</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>[характеристики с карточки — через |]</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>[слоган]</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,8 | Диаметр вводимой трубки, мм: 12,8 | Рабочая длина, мм: 1650 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 145</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Aohua</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Цена по запросу</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Строка-плейсхолдер. Реальные товары заполняются по карточкам medford.ru (ожидаются). Бренды из SERP: Pentax, Fujinon (Fujifilm), Olympus</t>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_ES_550T</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_es_550t</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape ЕС-550Т</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_es_550t/</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>12,0</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,0 | Диаметр вводимой трубки, мм: 12,5 | Рабочая длина, мм: 1700 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_SERII_EC_430</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_serii_ec_430</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape серии EC-430</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_serii_ec_430/</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_500</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_500</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-500</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_500/</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,5 | Диаметр вводимой трубки, мм: 12,5 | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_430T</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_430t</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-430T</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_430t/</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>12,0</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>12,0</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,0 | Диаметр вводимой трубки, мм: 12,0 | Рабочая длина, мм: 1700 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_EC_380FKP</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_pentax_ec_380fkp</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax EC-380FKp</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_pentax_ec_380fkp/</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр вводимой трубки, мм: 13,2 | Рабочая длина, мм: 1500 | Глубина резкости, мм: 3-100</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_550L_T</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_550l_t</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-550L/T</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_550l_t/</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,9 | Рабочая длина, мм: 1700 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_EC38_V10CM</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_pentax_ec38_v10cm</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax EC38-V10cM</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_pentax_ec38_v10cm/</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 13,2 | Диаметр вводимой трубки, мм: 13,2 | Рабочая длина, мм: 1300 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_MAGNIVIEW_EC_3890LZI</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_pentax_magniview_ec_3890lzi</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax MagniView EC‑3890LZi</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_pentax_magniview_ec_3890lzi/</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>13,0</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>4-100</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 13,0 | Диаметр вводимой трубки, мм: 13,2 | Рабочая длина, мм: 1700 | Глубина резкости, мм: 4-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_EC_3490LK</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_pentax_ec_3490lk</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax EC-3490LK</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_pentax_ec_3490lk/</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>11,6</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>11,5</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 11,5 | Диаметр вводимой трубки, мм: 11,6 | Рабочая длина, мм: 1700 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_330T</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_330t</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-330T</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_330t/</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>120º</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,9 | Диаметр вводимой трубки, мм: 12,9 | Рабочая длина, мм: 1600 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 120º</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_500T</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_500t</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-500T</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_500t/</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>1680</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,5 | Диаметр вводимой трубки, мм: 12,5 | Рабочая длина, мм: 1680 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_OLYMPUS_CF_HQ190L_I</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_olympus_cf_hq190l_i</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Olympus CF-HQ190L/I</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>240</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_olympus_cf_hq190l_i/</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>12,8</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>1330</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>5-100</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>170°</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,8 | Диаметр вводимой трубки, мм: 13,2 | Рабочая длина, мм: 1330 | Глубина резкости, мм: 5-100 | Угол поля зрения, °: 170°</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Olympus</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_550</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_550</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-550</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_550/</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>12,5</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>12,0</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,0 | Диаметр вводимой трубки, мм: 12,5 | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_FUJIFILM_EC_740TM</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_fujifilm_ec_740tm</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Fujifilm EC-740TM</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>260</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_fujifilm_ec_740tm/</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Fujifilm</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>10,7</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>9,8</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>1330</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 9,8 | Диаметр вводимой трубки, мм: 10,7 | Рабочая длина, мм: 1330 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Fujifilm</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_500L</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_500l</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-500L</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_500l/</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,9 | Диаметр вводимой трубки, мм: 12,9 | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_EC38_I10F2</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_pentax_ec38_i10f2</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax EC38-i10F2</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_pentax_ec38_i10f2/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>4-100</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>140°</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 13,2 | Диаметр вводимой трубки, мм: 13,2 | Рабочая длина, мм: 1500 | Глубина резкости, мм: 4-100 | Угол поля зрения, °: 140°</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_330</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_330</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-330</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>290</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_330/</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>120º</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,9 | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 120º</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_550L</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>videokolonoskop_sonoscape_ec_550l</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-550L</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>https://medford.ru/catalog/gibkaya_endoskopiya/endoskopy/kolonoskopy/videokolonoskop_sonoscape_ec_550l/</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Колоноскоп</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>3-100</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>уточнять</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>Тип оборудования: Колоноскоп | Диаметр дистального конца, мм: 12,9 | Рабочая длина, мм: 1350 | Глубина резкости, мм: 3-100 | Угол поля зрения, °: 140</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>Цена по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>20 товаров — реальный каталог medford.ru (все «Цена по запросу»). Характеристики — с карточек. Уточнить: страна, статус РУ, гарантия, инструментальный канал.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3682,7 +5636,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Для эндоскопических отделений и проктологии чаще всего выбирают видеоколоноскопы Pentax, Fujinon и Olympus — они дают чёткое HD-изображение и совместимы с большинством видеопроцессоров. Фиброколоноскопы остаются бюджетным решением для кабинетов с базовым потоком исследований. При подборе смотрят на рабочую длину и диаметр вводимой части, угол изгиба дистального конца и диаметр инструментального канала — от них зависят и диагностика, и лечебные манипуляции: полипэктомия, биопсия, остановка кровотечений.</t>
+          <t>Для эндоскопических отделений и проктологии сегодня выбирают видеоколоноскопы — они дают чёткое HD-изображение и совместимы с большинством видеопроцессоров. В нашем каталоге представлены SonoScape, Pentax, Olympus, Fujifilm и Aohua. При подборе смотрят на рабочую длину (обычно 1300–1700 мм) и диаметр вводимой части, глубину резкости и угол поля зрения, а также диаметр инструментального канала — от него зависят лечебные манипуляции: полипэктомия, биопсия, остановка кровотечений. Фиброколоноскопы остаются бюджетным решением для кабинетов с базовым потоком исследований.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Колоноскопы: trim hero footer and remove expert experience line
Remove delivery/warranty/company-license sentence from hero and the
'опыт [N лет]' experience mention from the expert block (applies to all
future category files too).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_kolonoskopy.xlsx
+++ b/medford_kolonoskopy.xlsx
@@ -2110,7 +2110,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Видеоколоноскопы для эндоскопических отделений и проктологии: диагностика толстой кишки, биопсия и лечебные манипуляции (полипэктомия, остановка кровотечений). В каталоге модели SonoScape, Pentax, Olympus, Fujifilm и Aohua. Доставка по России, монтаж и ввод в эксплуатацию, обучение персонала, гарантия и сервис. ООО «Медфорд» работает с 2009 года, лицензия Росздравнадзора ФС-99-04-000387 (ТОМИ).</t>
+          <t>Видеоколоноскопы для эндоскопических отделений и проктологии: диагностика толстой кишки, биопсия и лечебные манипуляции (полипэктомия, остановка кровотечений). В каталоге модели SonoScape, Pentax, Olympus, Fujifilm и Aohua.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Руководитель направления медтехники, Medford · опыт [N лет]</t>
+          <t>Руководитель направления медтехники, Medford</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Колоноскопы: add 07_RATING (top-5 from catalog products)
Build rating from the 20 catalog products, grounded in market reviews
(premium trio Olympus/Pentax/Fujifilm + value SonoScape) and specs (view
angle, optical zoom, distal diameter). Enable the RATING block.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Rw9dvcAKokoAsKsBSt35U
</commit_message>
<xml_diff>
--- a/medford_kolonoskopy.xlsx
+++ b/medford_kolonoskopy.xlsx
@@ -2498,13 +2498,17 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Рейтинг видеоколоноскопов 2026</t>
+        </is>
+      </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr">
         <is>
@@ -2513,7 +2517,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Отключён: ждём карточки товаров</t>
+          <t>Строки в 07_RATING</t>
         </is>
       </c>
     </row>
@@ -6299,25 +6303,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>07_RATING — Рейтинг (отключён, ждём карточки)</t>
+          <t>07_RATING — Рейтинг видеоколоноскопов 2026</t>
         </is>
       </c>
     </row>
@@ -6364,10 +6371,25 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>PROPERTY_BRAND</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>PROPERTY_RATING_POSITION</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_RATING_STARS</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTY_RATING_TAG</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>PROPERTY_NOTE</t>
         </is>
@@ -6384,15 +6406,15 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>[Модель]</t>
+          <t>Видеоколоноскоп Olympus CF-HQ190L/I</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -6407,21 +6429,277 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>[XML_ID]</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="n">
+          <t>VIDEOKOLONOSKOP_OLYMPUS_CF_HQ190L_I</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Заполнить после получения карточек товаров</t>
+      <c r="K4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Экспертный — обзор 170°</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Максимальный в каталоге угол поля зрения 170°; премиум-класс «большой тройки» (Olympus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>RATE_02</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax MagniView EC‑3890LZi</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>RATING</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_MAGNIVIEW_EC_3890LZI</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>С оптическим увеличением</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Технология MagniView (оптическое увеличение) для детальной диагностики слизистой</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>RATE_03</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Fujifilm EC-740TM</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>RATING</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_FUJIFILM_EC_740TM</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Fujifilm</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Самый тонкий — 9,8 мм</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Наименьший диаметр дистального конца (9,8 мм) — комфорт введения; премиум «большой тройки»</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>RATE_04</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп Pentax EC38-V10cM</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>RATING</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_PENTAX_EC38_V10CM</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Pentax</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Оптимум для клиники</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Сбалансированное решение премиум-бренда для современных клиник (по обзорам рынка)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>RATE_05</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Видеоколоноскоп SonoScape EC-500T</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>kolonoskopy</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>RATING</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>VIDEOKOLONOSKOP_SONOSCAPE_EC_500T</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>SonoScape</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Цена/качество</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Популярная HD-модель доступного сегмента; SonoScape и Aohua — бюджетная альтернатива «большой тройке»</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Рейтинг составлен по каталогу medford.ru: премиальная «большая тройка» (Olympus, Pentax, Fujifilm) + доступный сегмент (SonoScape, Aohua), с учётом характеристик (угол обзора, оптическое увеличение, диаметр) и обзоров рынка. Не является клиническим сравнением; звёзды — экспертная оценка тира.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>